<commit_message>
Logbuch um Aktivierungsfkt. + Skalierung ergänzt; Ansatz Lernrate bestimmen gesetzt
</commit_message>
<xml_diff>
--- a/results/Auswertung_Zusammenhang_Aktivierungsfunktion_Skalierung.xlsx
+++ b/results/Auswertung_Zusammenhang_Aktivierungsfunktion_Skalierung.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felixhollfoth/Documents/Uni/JLU/2. Semester/KI I/Projekt KI I Neu/ki-308/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9EFC218A-1A48-7241-8F09-499D1EDA5612}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EACFF784-D3DB-C246-98EA-6D25451F8E01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14520" yWindow="0" windowWidth="14280" windowHeight="18000" xr2:uid="{6AE51630-ABAF-EA4A-B486-091D5CE52967}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{6AE51630-ABAF-EA4A-B486-091D5CE52967}"/>
   </bookViews>
   <sheets>
     <sheet name="R^2 ja nach Akt. Und scaling " sheetId="1" r:id="rId1"/>
     <sheet name="Vergleich Skalierungen" sheetId="2" r:id="rId2"/>
+    <sheet name="LearningRate" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="28">
   <si>
     <t>Aktivierungsfunktion</t>
   </si>
@@ -78,9 +79,6 @@
     <t>Durchschnitt</t>
   </si>
   <si>
-    <t>=&gt; Manchmal Normal am besten aber häufig ist Standard am besten</t>
-  </si>
-  <si>
     <t>Differenz zwischen Train und Test Score:</t>
   </si>
   <si>
@@ -111,16 +109,19 @@
     <t>Mittelwert über die Aktivierungsfunktionen</t>
   </si>
   <si>
-    <t>=&gt; Modell macht einige Ausreißerfehler, da RMSE um circa 15% größer ist als MAE</t>
+    <t>Selu ist bester Kanditat aber nicht Haushoch überlegen &lt; 1 % gegenüber anderen Aktivierungsfunktionen</t>
   </si>
   <si>
-    <t>=&gt; Selu ist bester Kanditat aber nicht Haushoch überlegen &lt; 1 % gegenüber anderen Aktivierungsfunktionen</t>
+    <t>Selu lässt negative Werte zu und ist glatter als Relu, was einen stabileren Gradienten erzeugen kann</t>
   </si>
   <si>
-    <t>=&gt; Selu ist perfekt gegen nicht Normalverteilte Daten (Hier schiefe Verteilungen, Außreißer (manche noch vorhanden, unterschiedliche skalen)</t>
+    <t>Selu ist perfekt gegen nicht Normalverteilte Daten (Hier schiefe Verteilungen, Außreißer (manche noch vorhanden, unterschiedliche skalen)</t>
   </si>
   <si>
-    <t>=&gt; Selu lässt negative Werte zu und ist glatter als Relu, was einen stabileren Gradienten erzeugen kann</t>
+    <t>Relu und tanh neigen bereits zum overfitten (4 bis 6 % unterschied)</t>
+  </si>
+  <si>
+    <t>Selu danach am besten mit 2 % Unterschied</t>
   </si>
 </sst>
 </file>
@@ -177,9 +178,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -195,6 +196,1335 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="de-DE"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="de-DE"/>
+              <a:t>Testscore in Abhängigkeit der Lernrate</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.3224114578270309"/>
+          <c:y val="3.6553521046697124E-2"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="de-DE"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>LearningRate!$B$2:$B$51</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="50"/>
+                <c:pt idx="0">
+                  <c:v>1E-3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.1836734693877499E-3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.36734693877551E-3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.5510204081632499E-3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.734693877551E-3</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.9183673469387499E-3</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2.1020408163264998E-3</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2.2857142857142499E-3</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2.469387755102E-3</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2.6530612244897501E-3</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2.8367346938775002E-3</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>3.0204081632652499E-3</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>3.204081632653E-3</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>3.3877551020407501E-3</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>3.5714285714285002E-3</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>3.7551020408162499E-3</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>3.938775510204E-3</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>4.1224489795917496E-3</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>4.3061224489795002E-3</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>4.4897959183672499E-3</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>4.6734693877550004E-3</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>4.8571428571427501E-3</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>5.0408163265304997E-3</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>5.2244897959182503E-3</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>5.4081632653059999E-3</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>5.5918367346937496E-3</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>5.7755102040815002E-3</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>5.9591836734692498E-3</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>6.1428571428570004E-3</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>6.32653061224475E-3</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>6.5102040816324997E-3</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>6.6938775510202502E-3</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>6.8775510204079999E-3</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>7.0612244897957496E-3</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>7.2448979591835001E-3</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>7.4285714285712498E-3</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>7.6122448979590003E-3</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>7.79591836734675E-3</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>7.9795918367345006E-3</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>8.1632653061222502E-3</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>8.3469387755099999E-3</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>8.5306122448977496E-3</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>8.7142857142854906E-3</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>8.8979591836732402E-3</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>9.0816326530610003E-3</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>9.26530612244875E-3</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>9.4489795918364997E-3</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>9.6326530612242407E-3</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>9.8163265306119903E-3</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>9.99999999999974E-3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>LearningRate!$C$2:$C$51</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="50"/>
+                <c:pt idx="0">
+                  <c:v>0.75049999999999994</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.75229999999999997</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.74980000000000002</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.75360000000000005</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.72929999999999995</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.75829999999999997</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.74650000000000005</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.76080000000000003</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.74209999999999998</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.74929999999999997</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.71919999999999995</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.74380000000000002</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.75249999999999995</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.74650000000000005</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.75480000000000003</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.76190000000000002</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.74480000000000002</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.74309999999999998</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.75170000000000003</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.74919999999999998</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.75280000000000002</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>0.74299999999999999</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>0.75239999999999996</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>0.755</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>0.76239999999999997</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>0.75739999999999996</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>0.75509999999999999</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>0.74650000000000005</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>0.75309999999999999</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>0.75180000000000002</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>0.75780000000000003</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>0.754</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>0.7429</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>0.74099999999999999</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>0.74890000000000001</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>0.73770000000000002</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>0.75319999999999998</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>0.75290000000000001</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>0.75219999999999998</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>0.75949999999999995</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>0.72840000000000005</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>0.74409999999999998</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>0.747</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>0.75970000000000004</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>0.74470000000000003</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>0.74709999999999999</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>0.7429</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>0.72719999999999996</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>0.74770000000000003</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>0.7177</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-0837-5B49-8A66-73A0608C4ABD}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1939584560"/>
+        <c:axId val="1939586688"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1939584560"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="de-DE"/>
+                  <a:t>Lernrate</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="de-DE"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="de-DE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1939586688"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1939586688"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="de-DE"/>
+                  <a:t>R^2 Test Score</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="de-DE"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="de-DE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1939584560"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="de-DE"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.78740157499999996" l="0.7" r="0.7" t="0.78740157499999996" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>768350</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>12700</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>190500</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Diagramm 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9FA3E818-F3C1-9943-C344-B34B9743B9E8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -514,7 +1844,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E47E986-7593-8543-8F73-C13F2CFBBC88}">
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="18.5" bestFit="1" customWidth="1"/>
@@ -546,18 +1876,18 @@
       <c r="B3" t="s">
         <v>5</v>
       </c>
-      <c r="C3">
-        <v>0.78469999999999995</v>
-      </c>
-      <c r="D3">
-        <v>0.77980000000000005</v>
+      <c r="C3" s="2">
+        <v>-0.14000000000000001</v>
+      </c>
+      <c r="D3" s="3">
+        <v>0.81710000000000005</v>
       </c>
       <c r="E3">
-        <v>0.77729999999999999</v>
+        <v>0.78559999999999997</v>
       </c>
       <c r="F3" s="2">
         <f>AVERAGE(C3:E3)</f>
-        <v>0.78060000000000007</v>
+        <v>0.48756666666666665</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -565,17 +1895,17 @@
         <v>6</v>
       </c>
       <c r="C4">
-        <v>0.77349999999999997</v>
-      </c>
-      <c r="D4">
-        <v>0.78449999999999998</v>
+        <v>0.30599999999999999</v>
+      </c>
+      <c r="D4" s="3">
+        <v>0.80449999999999999</v>
       </c>
       <c r="E4">
-        <v>0.7782</v>
+        <v>0.74929999999999997</v>
       </c>
       <c r="F4" s="2">
         <f t="shared" ref="F4:F8" si="0">AVERAGE(C4:E4)</f>
-        <v>0.77873333333333328</v>
+        <v>0.61993333333333334</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -583,56 +1913,54 @@
         <v>7</v>
       </c>
       <c r="C5">
-        <v>0.78380000000000005</v>
-      </c>
-      <c r="D5">
-        <v>0.77429999999999999</v>
+        <v>0.56930000000000003</v>
+      </c>
+      <c r="D5" s="3">
+        <v>0.76429999999999998</v>
       </c>
       <c r="E5">
-        <v>0.77869999999999995</v>
+        <v>0.68520000000000003</v>
       </c>
       <c r="F5" s="2">
         <f t="shared" si="0"/>
-        <v>0.77893333333333337</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>13</v>
-      </c>
+        <v>0.67293333333333338</v>
+      </c>
+      <c r="G5" s="4"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>8</v>
       </c>
       <c r="C6">
-        <v>0.77939999999999998</v>
-      </c>
-      <c r="D6">
-        <v>0.78320000000000001</v>
+        <v>0.56230000000000002</v>
+      </c>
+      <c r="D6" s="3">
+        <v>0.76739999999999997</v>
       </c>
       <c r="E6">
-        <v>0.78069999999999995</v>
+        <v>0.72450000000000003</v>
       </c>
       <c r="F6" s="2">
         <f t="shared" si="0"/>
-        <v>0.78110000000000002</v>
+        <v>0.6847333333333333</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="3">
-        <v>0.7792</v>
+      <c r="C7" s="5">
+        <v>0.23910000000000001</v>
       </c>
       <c r="D7" s="3">
-        <v>0.78900000000000003</v>
-      </c>
-      <c r="E7" s="3">
-        <v>0.7873</v>
-      </c>
-      <c r="F7" s="4">
+        <v>0.77810000000000001</v>
+      </c>
+      <c r="E7" s="5">
+        <v>0.75460000000000005</v>
+      </c>
+      <c r="F7" s="6">
         <f t="shared" si="0"/>
-        <v>0.78516666666666668</v>
+        <v>0.59060000000000012</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -640,17 +1968,17 @@
         <v>10</v>
       </c>
       <c r="C8">
-        <v>0.77949999999999997</v>
-      </c>
-      <c r="D8">
-        <v>0.78259999999999996</v>
+        <v>-0.59030000000000005</v>
+      </c>
+      <c r="D8" s="3">
+        <v>0.79049999999999998</v>
       </c>
       <c r="E8">
-        <v>0.7782</v>
+        <v>0.7671</v>
       </c>
       <c r="F8" s="2">
         <f t="shared" si="0"/>
-        <v>0.78010000000000002</v>
+        <v>0.32243333333333329</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -680,17 +2008,17 @@
         <v>5</v>
       </c>
       <c r="C12">
-        <v>0.75780000000000003</v>
+        <v>-0.15040000000000001</v>
       </c>
       <c r="D12">
-        <v>0.75549999999999995</v>
-      </c>
-      <c r="E12">
-        <v>0.75429999999999997</v>
+        <v>0.75609999999999999</v>
+      </c>
+      <c r="E12" s="3">
+        <v>0.76180000000000003</v>
       </c>
       <c r="F12" s="2">
         <f>AVERAGE(C12:E12)</f>
-        <v>0.75586666666666658</v>
+        <v>0.45583333333333337</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -698,17 +2026,17 @@
         <v>6</v>
       </c>
       <c r="C13">
-        <v>0.75309999999999999</v>
-      </c>
-      <c r="D13">
-        <v>0.76249999999999996</v>
+        <v>0.309</v>
+      </c>
+      <c r="D13" s="3">
+        <v>0.76680000000000004</v>
       </c>
       <c r="E13">
-        <v>0.75609999999999999</v>
+        <v>0.74050000000000005</v>
       </c>
       <c r="F13" s="2">
         <f t="shared" ref="F13:F17" si="1">AVERAGE(C13:E13)</f>
-        <v>0.75723333333333331</v>
+        <v>0.60543333333333338</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -716,79 +2044,77 @@
         <v>7</v>
       </c>
       <c r="C14">
-        <v>0.76119999999999999</v>
-      </c>
-      <c r="D14">
-        <v>0.75239999999999996</v>
+        <v>0.56889999999999996</v>
+      </c>
+      <c r="D14" s="3">
+        <v>0.75290000000000001</v>
       </c>
       <c r="E14">
-        <v>0.75849999999999995</v>
+        <v>0.67859999999999998</v>
       </c>
       <c r="F14" s="2">
         <f t="shared" si="1"/>
-        <v>0.75736666666666663</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>13</v>
-      </c>
+        <v>0.66679999999999995</v>
+      </c>
+      <c r="G14" s="4"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B15" t="s">
         <v>8</v>
       </c>
       <c r="C15">
-        <v>0.75680000000000003</v>
-      </c>
-      <c r="D15">
-        <v>0.76200000000000001</v>
+        <v>0.55900000000000005</v>
+      </c>
+      <c r="D15" s="3">
+        <v>0.74790000000000001</v>
       </c>
       <c r="E15">
-        <v>0.75480000000000003</v>
+        <v>0.71650000000000003</v>
       </c>
       <c r="F15" s="2">
         <f t="shared" si="1"/>
-        <v>0.75786666666666669</v>
+        <v>0.67446666666666666</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C16" s="3">
-        <v>0.76119999999999999</v>
+      <c r="C16" s="5">
+        <v>0.23150000000000001</v>
       </c>
       <c r="D16" s="3">
-        <v>0.76749999999999996</v>
-      </c>
-      <c r="E16" s="3">
-        <v>0.76070000000000004</v>
-      </c>
-      <c r="F16" s="4">
+        <v>0.75770000000000004</v>
+      </c>
+      <c r="E16" s="5">
+        <v>0.74619999999999997</v>
+      </c>
+      <c r="F16" s="6">
         <f t="shared" si="1"/>
-        <v>0.76313333333333333</v>
+        <v>0.57846666666666668</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B17" t="s">
         <v>10</v>
       </c>
-      <c r="C17">
-        <v>0.75609999999999999</v>
-      </c>
-      <c r="D17">
-        <v>0.76219999999999999</v>
-      </c>
-      <c r="E17">
-        <v>0.75329999999999997</v>
+      <c r="C17" s="5">
+        <v>-0.58919999999999995</v>
+      </c>
+      <c r="D17" s="3">
+        <v>0.75639999999999996</v>
+      </c>
+      <c r="E17" s="5">
+        <v>0.75409999999999999</v>
       </c>
       <c r="F17" s="2">
         <f t="shared" si="1"/>
-        <v>0.75719999999999998</v>
+        <v>0.30709999999999998</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
@@ -804,9 +2130,7 @@
       <c r="E20" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F20" s="1" t="s">
-        <v>12</v>
-      </c>
+      <c r="F20" s="1"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
@@ -814,20 +2138,17 @@
       </c>
       <c r="C21">
         <f>C3-C12</f>
-        <v>2.6899999999999924E-2</v>
+        <v>1.0399999999999993E-2</v>
       </c>
       <c r="D21">
         <f t="shared" ref="D21:F21" si="2">D3-D12</f>
-        <v>2.4300000000000099E-2</v>
+        <v>6.1000000000000054E-2</v>
       </c>
       <c r="E21">
         <f t="shared" si="2"/>
-        <v>2.300000000000002E-2</v>
-      </c>
-      <c r="F21" s="2">
-        <f t="shared" si="2"/>
-        <v>2.4733333333333496E-2</v>
-      </c>
+        <v>2.3799999999999932E-2</v>
+      </c>
+      <c r="F21" s="2"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B22" t="s">
@@ -835,20 +2156,17 @@
       </c>
       <c r="C22">
         <f t="shared" ref="C22:F26" si="3">C4-C13</f>
-        <v>2.0399999999999974E-2</v>
+        <v>-3.0000000000000027E-3</v>
       </c>
       <c r="D22">
         <f t="shared" si="3"/>
-        <v>2.200000000000002E-2</v>
+        <v>3.7699999999999956E-2</v>
       </c>
       <c r="E22">
         <f t="shared" si="3"/>
-        <v>2.2100000000000009E-2</v>
-      </c>
-      <c r="F22" s="2">
-        <f t="shared" si="3"/>
-        <v>2.1499999999999964E-2</v>
-      </c>
+        <v>8.799999999999919E-3</v>
+      </c>
+      <c r="F22" s="2"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
@@ -856,20 +2174,17 @@
       </c>
       <c r="C23">
         <f t="shared" si="3"/>
-        <v>2.2600000000000064E-2</v>
+        <v>4.0000000000006697E-4</v>
       </c>
       <c r="D23">
         <f t="shared" si="3"/>
-        <v>2.1900000000000031E-2</v>
+        <v>1.1399999999999966E-2</v>
       </c>
       <c r="E23">
         <f t="shared" si="3"/>
-        <v>2.0199999999999996E-2</v>
-      </c>
-      <c r="F23" s="2">
-        <f t="shared" si="3"/>
-        <v>2.1566666666666734E-2</v>
-      </c>
+        <v>6.6000000000000503E-3</v>
+      </c>
+      <c r="F23" s="2"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
@@ -877,41 +2192,35 @@
       </c>
       <c r="C24">
         <f t="shared" si="3"/>
-        <v>2.2599999999999953E-2</v>
+        <v>3.2999999999999696E-3</v>
       </c>
       <c r="D24">
         <f t="shared" si="3"/>
-        <v>2.1199999999999997E-2</v>
+        <v>1.9499999999999962E-2</v>
       </c>
       <c r="E24">
         <f t="shared" si="3"/>
-        <v>2.5899999999999923E-2</v>
-      </c>
-      <c r="F24" s="2">
-        <f t="shared" si="3"/>
-        <v>2.3233333333333328E-2</v>
-      </c>
+        <v>8.0000000000000071E-3</v>
+      </c>
+      <c r="F24" s="2"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C25">
         <f t="shared" si="3"/>
-        <v>1.8000000000000016E-2</v>
+        <v>7.5999999999999956E-3</v>
       </c>
       <c r="D25">
         <f t="shared" si="3"/>
-        <v>2.1500000000000075E-2</v>
+        <v>2.0399999999999974E-2</v>
       </c>
       <c r="E25">
         <f t="shared" si="3"/>
-        <v>2.6599999999999957E-2</v>
-      </c>
-      <c r="F25" s="2">
-        <f t="shared" si="3"/>
-        <v>2.2033333333333349E-2</v>
-      </c>
+        <v>8.4000000000000741E-3</v>
+      </c>
+      <c r="F25" s="2"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B26" t="s">
@@ -919,35 +2228,45 @@
       </c>
       <c r="C26">
         <f t="shared" si="3"/>
-        <v>2.3399999999999976E-2</v>
+        <v>-1.1000000000001009E-3</v>
       </c>
       <c r="D26">
         <f t="shared" si="3"/>
-        <v>2.0399999999999974E-2</v>
+        <v>3.4100000000000019E-2</v>
       </c>
       <c r="E26">
         <f t="shared" si="3"/>
-        <v>2.4900000000000033E-2</v>
-      </c>
-      <c r="F26" s="2">
-        <f t="shared" si="3"/>
-        <v>2.2900000000000031E-2</v>
-      </c>
+        <v>1.3000000000000012E-2</v>
+      </c>
+      <c r="F26" s="2"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A28" s="5" t="s">
+      <c r="A28" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A29" s="4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A29" s="5" t="s">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A30" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A32" s="4" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A30" s="5" t="s">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A33" s="4" t="s">
         <v>27</v>
       </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A34" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -961,83 +2280,460 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="2">
-        <v>0.78</v>
-      </c>
-      <c r="D3">
-        <v>0.75770000000000004</v>
-      </c>
-      <c r="E3">
-        <v>0.32490000000000002</v>
-      </c>
-      <c r="F3">
-        <v>0.46910000000000002</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="C3" s="2"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4">
-        <v>0.78220000000000001</v>
-      </c>
-      <c r="D4">
-        <v>0.76039999999999996</v>
-      </c>
-      <c r="E4">
-        <v>0.32450000000000001</v>
-      </c>
-      <c r="F4">
-        <v>0.4667</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5">
-        <v>0.78010000000000002</v>
-      </c>
-      <c r="D5">
-        <v>0.75629999999999997</v>
-      </c>
-      <c r="E5">
-        <v>0.32929999999999998</v>
-      </c>
-      <c r="F5">
-        <v>0.47060000000000002</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" s="5" t="s">
-        <v>24</v>
-      </c>
+      <c r="A7" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8F5FF89-2000-F741-863F-4FDE338F0174}">
+  <dimension ref="B2:C51"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="22.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B2">
+        <v>1E-3</v>
+      </c>
+      <c r="C2">
+        <v>0.75049999999999994</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B3">
+        <v>1.1836734693877499E-3</v>
+      </c>
+      <c r="C3">
+        <v>0.75229999999999997</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B4">
+        <v>1.36734693877551E-3</v>
+      </c>
+      <c r="C4">
+        <v>0.74980000000000002</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B5">
+        <v>1.5510204081632499E-3</v>
+      </c>
+      <c r="C5">
+        <v>0.75360000000000005</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B6">
+        <v>1.734693877551E-3</v>
+      </c>
+      <c r="C6">
+        <v>0.72929999999999995</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B7">
+        <v>1.9183673469387499E-3</v>
+      </c>
+      <c r="C7">
+        <v>0.75829999999999997</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B8">
+        <v>2.1020408163264998E-3</v>
+      </c>
+      <c r="C8">
+        <v>0.74650000000000005</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B9">
+        <v>2.2857142857142499E-3</v>
+      </c>
+      <c r="C9">
+        <v>0.76080000000000003</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B10">
+        <v>2.469387755102E-3</v>
+      </c>
+      <c r="C10">
+        <v>0.74209999999999998</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B11">
+        <v>2.6530612244897501E-3</v>
+      </c>
+      <c r="C11">
+        <v>0.74929999999999997</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B12">
+        <v>2.8367346938775002E-3</v>
+      </c>
+      <c r="C12">
+        <v>0.71919999999999995</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B13">
+        <v>3.0204081632652499E-3</v>
+      </c>
+      <c r="C13">
+        <v>0.74380000000000002</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B14">
+        <v>3.204081632653E-3</v>
+      </c>
+      <c r="C14">
+        <v>0.75249999999999995</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B15">
+        <v>3.3877551020407501E-3</v>
+      </c>
+      <c r="C15">
+        <v>0.74650000000000005</v>
+      </c>
+    </row>
+    <row r="16" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B16">
+        <v>3.5714285714285002E-3</v>
+      </c>
+      <c r="C16">
+        <v>0.75480000000000003</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B17">
+        <v>3.7551020408162499E-3</v>
+      </c>
+      <c r="C17">
+        <v>0.76190000000000002</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B18">
+        <v>3.938775510204E-3</v>
+      </c>
+      <c r="C18">
+        <v>0.74480000000000002</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B19">
+        <v>4.1224489795917496E-3</v>
+      </c>
+      <c r="C19">
+        <v>0.74309999999999998</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B20">
+        <v>4.3061224489795002E-3</v>
+      </c>
+      <c r="C20">
+        <v>0.75170000000000003</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B21">
+        <v>4.4897959183672499E-3</v>
+      </c>
+      <c r="C21">
+        <v>0.74919999999999998</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B22">
+        <v>4.6734693877550004E-3</v>
+      </c>
+      <c r="C22">
+        <v>0.75280000000000002</v>
+      </c>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B23">
+        <v>4.8571428571427501E-3</v>
+      </c>
+      <c r="C23">
+        <v>0.74299999999999999</v>
+      </c>
+    </row>
+    <row r="24" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B24">
+        <v>5.0408163265304997E-3</v>
+      </c>
+      <c r="C24">
+        <v>0.75239999999999996</v>
+      </c>
+    </row>
+    <row r="25" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B25">
+        <v>5.2244897959182503E-3</v>
+      </c>
+      <c r="C25">
+        <v>0.755</v>
+      </c>
+    </row>
+    <row r="26" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B26">
+        <v>5.4081632653059999E-3</v>
+      </c>
+      <c r="C26">
+        <v>0.76239999999999997</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B27">
+        <v>5.5918367346937496E-3</v>
+      </c>
+      <c r="C27">
+        <v>0.75739999999999996</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B28">
+        <v>5.7755102040815002E-3</v>
+      </c>
+      <c r="C28">
+        <v>0.75509999999999999</v>
+      </c>
+    </row>
+    <row r="29" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B29">
+        <v>5.9591836734692498E-3</v>
+      </c>
+      <c r="C29">
+        <v>0.74650000000000005</v>
+      </c>
+    </row>
+    <row r="30" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B30">
+        <v>6.1428571428570004E-3</v>
+      </c>
+      <c r="C30">
+        <v>0.75309999999999999</v>
+      </c>
+    </row>
+    <row r="31" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B31">
+        <v>6.32653061224475E-3</v>
+      </c>
+      <c r="C31">
+        <v>0.75180000000000002</v>
+      </c>
+    </row>
+    <row r="32" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B32">
+        <v>6.5102040816324997E-3</v>
+      </c>
+      <c r="C32">
+        <v>0.75780000000000003</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B33">
+        <v>6.6938775510202502E-3</v>
+      </c>
+      <c r="C33">
+        <v>0.754</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B34">
+        <v>6.8775510204079999E-3</v>
+      </c>
+      <c r="C34">
+        <v>0.7429</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B35">
+        <v>7.0612244897957496E-3</v>
+      </c>
+      <c r="C35">
+        <v>0.74099999999999999</v>
+      </c>
+    </row>
+    <row r="36" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B36">
+        <v>7.2448979591835001E-3</v>
+      </c>
+      <c r="C36">
+        <v>0.74890000000000001</v>
+      </c>
+    </row>
+    <row r="37" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B37">
+        <v>7.4285714285712498E-3</v>
+      </c>
+      <c r="C37">
+        <v>0.73770000000000002</v>
+      </c>
+    </row>
+    <row r="38" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B38">
+        <v>7.6122448979590003E-3</v>
+      </c>
+      <c r="C38">
+        <v>0.75319999999999998</v>
+      </c>
+    </row>
+    <row r="39" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B39">
+        <v>7.79591836734675E-3</v>
+      </c>
+      <c r="C39">
+        <v>0.75290000000000001</v>
+      </c>
+    </row>
+    <row r="40" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B40">
+        <v>7.9795918367345006E-3</v>
+      </c>
+      <c r="C40">
+        <v>0.75219999999999998</v>
+      </c>
+    </row>
+    <row r="41" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B41">
+        <v>8.1632653061222502E-3</v>
+      </c>
+      <c r="C41">
+        <v>0.75949999999999995</v>
+      </c>
+    </row>
+    <row r="42" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B42">
+        <v>8.3469387755099999E-3</v>
+      </c>
+      <c r="C42">
+        <v>0.72840000000000005</v>
+      </c>
+    </row>
+    <row r="43" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B43">
+        <v>8.5306122448977496E-3</v>
+      </c>
+      <c r="C43">
+        <v>0.74409999999999998</v>
+      </c>
+    </row>
+    <row r="44" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B44">
+        <v>8.7142857142854906E-3</v>
+      </c>
+      <c r="C44">
+        <v>0.747</v>
+      </c>
+    </row>
+    <row r="45" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B45">
+        <v>8.8979591836732402E-3</v>
+      </c>
+      <c r="C45">
+        <v>0.75970000000000004</v>
+      </c>
+    </row>
+    <row r="46" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B46">
+        <v>9.0816326530610003E-3</v>
+      </c>
+      <c r="C46">
+        <v>0.74470000000000003</v>
+      </c>
+    </row>
+    <row r="47" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B47">
+        <v>9.26530612244875E-3</v>
+      </c>
+      <c r="C47">
+        <v>0.74709999999999999</v>
+      </c>
+    </row>
+    <row r="48" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B48">
+        <v>9.4489795918364997E-3</v>
+      </c>
+      <c r="C48">
+        <v>0.7429</v>
+      </c>
+    </row>
+    <row r="49" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B49">
+        <v>9.6326530612242407E-3</v>
+      </c>
+      <c r="C49">
+        <v>0.72719999999999996</v>
+      </c>
+    </row>
+    <row r="50" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B50">
+        <v>9.8163265306119903E-3</v>
+      </c>
+      <c r="C50">
+        <v>0.74770000000000003</v>
+      </c>
+    </row>
+    <row r="51" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B51">
+        <v>9.99999999999974E-3</v>
+      </c>
+      <c r="C51">
+        <v>0.7177</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Logbuch Verbesserungen bis einschließlich Eintrag 9
</commit_message>
<xml_diff>
--- a/results/Auswertung_Zusammenhang_Aktivierungsfunktion_Skalierung.xlsx
+++ b/results/Auswertung_Zusammenhang_Aktivierungsfunktion_Skalierung.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felixhollfoth/Documents/Uni/JLU/2. Semester/KI I/Projekt KI I Neu/ki-308/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DF0EE93-C277-F841-AA7E-BD7DB7BC8F48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D5CD62C-EE1D-BA4F-A1B8-E29E2521A0D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="3" xr2:uid="{6AE51630-ABAF-EA4A-B486-091D5CE52967}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" activeTab="3" xr2:uid="{6AE51630-ABAF-EA4A-B486-091D5CE52967}"/>
   </bookViews>
   <sheets>
     <sheet name="R^2 ja nach Akt. Und scaling " sheetId="1" r:id="rId1"/>
@@ -2765,6 +2765,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A49FA0A-7B07-404D-84E0-17E523C045F6}">
   <dimension ref="B2:F14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="13.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="2" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B2" t="s">

</xml_diff>